<commit_message>
Data for Kill-/Razesanity + Carracks
</commit_message>
<xml_diff>
--- a/docs/Logic Requirements/Ageipelago Saladin.xlsx
+++ b/docs/Logic Requirements/Ageipelago Saladin.xlsx
@@ -5,15 +5,21 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/BB6DD295C338E39F/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stefb\OneDrive\Desktop\Logic Requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="8_{3B7C1B1A-253A-4772-BD48-CE4AC1339EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EC11DFB-BCCE-49F4-A80A-5E7D2AB0343B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CD2FBCA-71C4-4512-BCD3-CF7D87603E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AEFAB4D2-F215-45BA-9EF6-82F1BCF340C6}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{AEFAB4D2-F215-45BA-9EF6-82F1BCF340C6}"/>
   </bookViews>
   <sheets>
     <sheet name="Saladin" sheetId="1" r:id="rId1"/>
+    <sheet name="An Arabian Knight" sheetId="2" r:id="rId2"/>
+    <sheet name="Lord of Arabia" sheetId="3" r:id="rId3"/>
+    <sheet name="The Horns of Hattin" sheetId="4" r:id="rId4"/>
+    <sheet name="The Siege of Jerusalem" sheetId="5" r:id="rId5"/>
+    <sheet name="Jihad!" sheetId="6" r:id="rId6"/>
+    <sheet name="The Lion and the Demon" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="188">
   <si>
     <t>The Lion and the Demon</t>
   </si>
@@ -951,85 +957,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-12 Men-at-Arms
-12 Knights
-1 Scout
-17 Crossbowmen
-2 Throwing Axemen
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Standard:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Identical to Moderate
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Hard:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-12 Men-at-Arms
-12 Knights
-1 Scout
-21 Crossbowmen
-2 Throwing Axemen
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Moderate:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
 4 Camel Riders
 13 Archers
 10 Mamelukes
@@ -1158,33 +1085,6 @@
       </rPr>
       <t xml:space="preserve">
 Identical to Standard</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Just added </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>the Pyramids</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> because… Why not?
-The only Ecplanation I've got for the Player 4 Army
-being bigger on Standard is that someone mixed up Standard and Moderate on Development…</t>
     </r>
   </si>
   <si>
@@ -1862,103 +1762,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Starting Units:
-2 Trebuchets
-2 Galleons
-2 Cannon Galleons
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Moderate:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Later:
-17 Elite Serjeants
-4 Siege Onagers
-4 Trebuchets
-6 Galleons
-3 Fire Ships
-4 Heavy Demolition Ships
-3 Cannon Galleons
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Standard:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Later:
-13 Elite Serjeants
-4 Siege Onagers
-6 Galleons
-3 Fire Ships
-4 Heavy Demolition Ships
-3 Cannon Galleons
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Hard:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Later:
-21 Elite Serjeants
-4 Siege Onagers
-4 Trebuchets
-6 Galleons
-3 Fire Ships
-4 Heavy Demolition Ships
-3 Cannon Galleons</t>
-    </r>
-  </si>
-  <si>
-    <r>
       <rPr>
         <b/>
         <sz val="14"/>
@@ -2041,26 +1844,462 @@
   </si>
   <si>
     <t>Starting Units:
-2 Galleons
-2 Fast Fire Ships
-1 Cannon Galleon
+4 Light Cavalry
 Later:
-4 Light Cavalry
-16 Galleons
-4 Demoliton Ships
-5 Elite Cannon Galleons</t>
+10 Champions
+10 Light Cavalry
+4 Onagers
+4 Trebuchets</t>
   </si>
   <si>
     <t>Starting Units:
 4 Paladins
+2 Siege Rams
+3 Bombard Cannons
 Later:
-10 Elite Teutonic Knights
-8 Paldins
-10 Capped Rams</t>
+10 Paladins
+6 Hand Cannoneers
+8 Bombard Cannons</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The Player needs to have unlocked Warships to defeat </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF24E7FC"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Genoese</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.
+The Player needs to have unlocked Wonders to build a Wonder.</t>
+    </r>
+  </si>
+  <si>
+    <t>No items required</t>
+  </si>
+  <si>
+    <t>Elite Skirmisher</t>
+  </si>
+  <si>
+    <t>Requires Dock</t>
+  </si>
+  <si>
+    <t>Galleon</t>
+  </si>
+  <si>
+    <t>War Galley</t>
+  </si>
+  <si>
+    <t>Guard Tower</t>
+  </si>
+  <si>
+    <t>Galley</t>
+  </si>
+  <si>
+    <t>Dock</t>
+  </si>
+  <si>
+    <t>Watch Tower</t>
+  </si>
+  <si>
+    <t>Outpost</t>
+  </si>
+  <si>
+    <t>Trebuchet</t>
+  </si>
+  <si>
+    <t>Fortified Wall</t>
+  </si>
+  <si>
+    <t>Stone Gate</t>
+  </si>
+  <si>
+    <t>Stone Wall</t>
+  </si>
+  <si>
+    <t>Light Cavalry</t>
+  </si>
+  <si>
+    <t>Castle</t>
+  </si>
+  <si>
+    <t>Blacksmith</t>
+  </si>
+  <si>
+    <t>Barracks</t>
+  </si>
+  <si>
+    <t>University</t>
+  </si>
+  <si>
+    <t>Mining Camp</t>
+  </si>
+  <si>
+    <t>Battering Ram</t>
+  </si>
+  <si>
+    <t>Monastery</t>
+  </si>
+  <si>
+    <t>Market</t>
+  </si>
+  <si>
+    <t>Monk</t>
+  </si>
+  <si>
+    <t>Archery Range</t>
+  </si>
+  <si>
+    <t>Mill</t>
+  </si>
+  <si>
+    <t>Scout Cavalry</t>
+  </si>
+  <si>
+    <t>Stable</t>
+  </si>
+  <si>
+    <t>Crossbowman</t>
+  </si>
+  <si>
+    <t>Town Center</t>
+  </si>
+  <si>
+    <t>Villager</t>
+  </si>
+  <si>
+    <t>Lumber Camp</t>
+  </si>
+  <si>
+    <t>Siege Workshop</t>
+  </si>
+  <si>
+    <t>Farm</t>
+  </si>
+  <si>
+    <t>Sheep</t>
+  </si>
+  <si>
+    <t>House</t>
+  </si>
+  <si>
+    <t>Deer</t>
+  </si>
+  <si>
+    <t>Destructible Buildings</t>
+  </si>
+  <si>
+    <t>Killable Units</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Just added </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>the Pyramids</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> because… Why not?
+The only Explanation I've got for the Player 4 Army
+being bigger on Standard is that someone mixed up Standard and Moderate on Development…</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Moderate:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+12 Men-at-Arms
+12 Knights
+1 Scout Cavalry
+17 Crossbowmen
+2 Throwing Axemen
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Standard:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Identical to Moderate
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hard:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+12 Men-at-Arms
+12 Knights
+1 Scout Cavalry
+21 Crossbowmen
+2 Throwing Axemen
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Man-at-Arms</t>
+  </si>
+  <si>
+    <t>Throwing Axeman</t>
+  </si>
+  <si>
+    <t>Knight</t>
+  </si>
+  <si>
+    <t>Archer</t>
+  </si>
+  <si>
+    <t>Camel Rider</t>
+  </si>
+  <si>
+    <t>Pikeman</t>
+  </si>
+  <si>
+    <t>Onager</t>
+  </si>
+  <si>
+    <t>Pavilion</t>
+  </si>
+  <si>
+    <t>Pavilion (Large)</t>
+  </si>
+  <si>
+    <t>Great Pyramid</t>
+  </si>
+  <si>
+    <t>Mosque</t>
+  </si>
+  <si>
+    <t>Barricade</t>
+  </si>
+  <si>
+    <t>Wild Camel</t>
+  </si>
+  <si>
+    <t>Skirmisher</t>
+  </si>
+  <si>
+    <t>Cavalier</t>
+  </si>
+  <si>
+    <t>Paladin</t>
+  </si>
+  <si>
+    <t>Mangonel</t>
+  </si>
+  <si>
+    <t>Reynald de Chatillon</t>
+  </si>
+  <si>
+    <t>Transport Ship</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Fire Ship
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(Not on Standard)</t>
+    </r>
+  </si>
+  <si>
+    <t>Requires Dock
+Only appears for a small Timeframe, maybe only consider for Hard Logic.</t>
+  </si>
+  <si>
+    <t>Trade Cart</t>
+  </si>
+  <si>
+    <t>Trade Cog</t>
+  </si>
+  <si>
+    <t>Fishing Ship</t>
+  </si>
+  <si>
+    <t>Palisade Wall</t>
+  </si>
+  <si>
+    <t>Trade Workshop</t>
+  </si>
+  <si>
+    <t>Monsatery</t>
+  </si>
+  <si>
+    <t>Scorpion</t>
+  </si>
+  <si>
+    <t>Man-at-Atms</t>
+  </si>
+  <si>
+    <t>Long Swordsman</t>
+  </si>
+  <si>
+    <t>Teutonic Knight</t>
+  </si>
+  <si>
+    <t>Master of the Templar</t>
+  </si>
+  <si>
+    <t>Halberdier</t>
+  </si>
+  <si>
+    <t>Arbalester</t>
+  </si>
+  <si>
+    <t>Cataphract</t>
+  </si>
+  <si>
+    <t>Elite Cataphract</t>
+  </si>
+  <si>
+    <t>Bombard Tower</t>
+  </si>
+  <si>
+    <t>Dome of the Rock</t>
+  </si>
+  <si>
+    <t>Destroying any of these is a Defeat Condition</t>
+  </si>
+  <si>
+    <t>Destroying this is a Defeat Condition</t>
+  </si>
+  <si>
+    <t>Fence</t>
+  </si>
+  <si>
+    <t>Wild Boar</t>
+  </si>
+  <si>
+    <t>Grey Wolf</t>
+  </si>
+  <si>
+    <t>Fast Fire Ship</t>
+  </si>
+  <si>
+    <t>Heavy Demolition Ship</t>
+  </si>
+  <si>
+    <t>Cannon Galleon</t>
+  </si>
+  <si>
+    <t>Heavy Camel Rider</t>
+  </si>
+  <si>
+    <t>Savar</t>
+  </si>
+  <si>
+    <t>Fire Ship</t>
+  </si>
+  <si>
+    <t>Elite Serjeant</t>
+  </si>
+  <si>
+    <t>Siege Onager</t>
+  </si>
+  <si>
+    <t>Keep</t>
+  </si>
+  <si>
+    <t>Fortified Gate</t>
+  </si>
+  <si>
+    <t>Wonder</t>
+  </si>
+  <si>
+    <t>Siege Ram</t>
+  </si>
+  <si>
+    <t>Bombard Cannon</t>
+  </si>
+  <si>
+    <t>Hand Cannoneer</t>
+  </si>
+  <si>
+    <t>Champion</t>
   </si>
   <si>
     <t>Starting Units:
-4 Chevalier
+4 Chavalier
 5 Elite Longbowmen
 2 Onagers
 Bad Neighbor
@@ -2072,56 +2311,157 @@
 3 Trebuchets</t>
   </si>
   <si>
-    <t>Starting Units:
-4 Light Cavalry
-Later:
-10 Champions
-10 Light Cavalry
-4 Onagers
-4 Trebuchets</t>
+    <t>Elite Longbowman</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scorpion </t>
+  </si>
+  <si>
+    <t>Bad Neighbor</t>
+  </si>
+  <si>
+    <t>God's Own Sling</t>
   </si>
   <si>
     <t>Starting Units:
 4 Paladins
-2 Siege Rams
-3 Bombard Cannons
 Later:
-10 Paladins
-6 Hand Cannoneers
-8 Bombard Cannons</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The Player needs to have unlocked Warships to defeat </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF24E7FC"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Genoese</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>.
-The Player needs to have unlocked Wonders to build a Wonder.</t>
-    </r>
+10 Elite Teutonic Knights
+8 Paladins
+10 Capped Rams</t>
+  </si>
+  <si>
+    <t>Elite Teutonic Knight</t>
+  </si>
+  <si>
+    <t>Capped Ram</t>
+  </si>
+  <si>
+    <t>Elite Cannon Galleon</t>
+  </si>
+  <si>
+    <t>Carrack</t>
+  </si>
+  <si>
+    <t>Starting Units:
+2 Galleons
+2 Fast Fire Ships
+1 Cannon Galleon
+Later:
+4 Light Cavalry
+16 Galleons
+4 Carracks
+5 Elite Cannon Galleons</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Starting Units:
+2 Trebuchets
+2 Galleons
+2 Cannon Galleons
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Moderate:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Later:
+17 Elite Serjeants
+4 Siege Onagers
+4 Trebuchets
+6 Galleons
+3 Fire Ships
+4 Carracks
+3 Cannon Galleons
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Standard:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Later:
+13 Elite Serjeants
+4 Siege Onagers
+6 Galleons
+3 Fire Ships
+4 Carracks
+3 Cannon Galleons
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hard:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Later:
+21 Elite Serjeants
+4 Siege Onagers
+4 Trebuchets
+6 Galleons
+3 Fire Ships
+4 Carracks
+3 Cannon Galleons</t>
+    </r>
+  </si>
+  <si>
+    <t>Mameluke</t>
+  </si>
+  <si>
+    <t>Pyramid</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="33" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2145,19 +2485,6 @@
     <font>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color rgb="FF3A3A3A"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color rgb="FF3A3A3A"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -2192,12 +2519,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="24"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="14"/>
@@ -2271,6 +2592,89 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="24"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="0" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF24E7FC"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFC000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFF00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2280,7 +2684,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -2368,11 +2772,59 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2386,12 +2838,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2401,13 +2847,119 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2733,7 +3285,7 @@
   <dimension ref="B2:Q9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="22.5703125" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" style="16" customWidth="1"/>
     <col min="3" max="3" width="24.85546875" customWidth="1"/>
     <col min="4" max="4" width="25.7109375" customWidth="1"/>
     <col min="5" max="5" width="31.140625" customWidth="1"/>
@@ -2753,7 +3305,7 @@
   <sheetData>
     <row r="2" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:17" ht="44.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="17" t="s">
         <v>17</v>
       </c>
       <c r="C3" s="4" t="s">
@@ -2771,77 +3323,77 @@
       <c r="G3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I3" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="J3" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="K3" s="10" t="s">
+      <c r="K3" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="L3" s="10" t="s">
+      <c r="L3" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="M3" s="10" t="s">
+      <c r="M3" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="N3" s="10" t="s">
+      <c r="N3" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="O3" s="10" t="s">
+      <c r="O3" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="P3" s="10" t="s">
+      <c r="P3" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="Q3" s="10" t="s">
+      <c r="Q3" s="8" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="4" spans="2:17" ht="282" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8" t="s">
+      <c r="G4" s="6"/>
+      <c r="H4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="J4" s="7" t="s">
+      <c r="I4" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="K4" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="L4" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="M4" s="7"/>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="7"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
     </row>
     <row r="5" spans="2:17" ht="319.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="18" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="3" t="s">
@@ -2859,25 +3411,25 @@
       <c r="I5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7" t="s">
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N5" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="M5" s="7" t="s">
+      <c r="O5" s="5"/>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="N5" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="O5" s="7"/>
-      <c r="P5" s="7"/>
-      <c r="Q5" s="7" t="s">
-        <v>57</v>
-      </c>
     </row>
     <row r="6" spans="2:17" ht="300.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="19" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="3" t="s">
@@ -2895,29 +3447,29 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="J6" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="M6" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="K6" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="L6" s="7" t="s">
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="M6" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="N6" s="7"/>
-      <c r="O6" s="7"/>
-      <c r="P6" s="7"/>
-      <c r="Q6" s="7" t="s">
-        <v>61</v>
-      </c>
     </row>
     <row r="7" spans="2:17" ht="394.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="18" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -2933,27 +3485,27 @@
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="K7" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="J7" s="7" t="s">
+      <c r="L7" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="K7" s="7" t="s">
+      <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="L7" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="7"/>
-      <c r="Q7" s="7" t="s">
-        <v>67</v>
-      </c>
     </row>
     <row r="8" spans="2:17" ht="409.6" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="18" t="s">
         <v>1</v>
       </c>
       <c r="C8" s="3" t="s">
@@ -2975,27 +3527,27 @@
       <c r="I8" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J8" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="K8" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="L8" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7" t="s">
+      <c r="J8" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="O8" s="7"/>
-      <c r="P8" s="7"/>
-      <c r="Q8" s="7" t="s">
+      <c r="K8" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="L8" s="5" t="s">
         <v>70</v>
       </c>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="O8" s="5"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="9" spans="2:17" ht="207" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="18" t="s">
         <v>0</v>
       </c>
       <c r="C9" s="3" t="s">
@@ -3017,31 +3569,2648 @@
       <c r="I9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J9" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="L9" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="M9" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="N9" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="O9" s="7" t="s">
+      <c r="J9" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="M9" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="O9" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5" t="s">
         <v>74</v>
-      </c>
-      <c r="P9" s="7"/>
-      <c r="Q9" s="7" t="s">
-        <v>80</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{853A5127-1C52-4219-B26B-767FBE00E695}">
+  <dimension ref="G1:L42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="8" width="22.5703125" customWidth="1"/>
+    <col min="11" max="12" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G3" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="L3" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G4" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K4" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G5" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K5" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G6" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K6" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G7" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G8" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K8" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G9" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K9" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G10" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K10" s="42" t="s">
+        <v>187</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G11" s="42" t="s">
+        <v>186</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K11" s="42" t="s">
+        <v>125</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G12" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K12" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G13" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="K13" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G14" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="K14" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="K15" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
+      <c r="K16" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
+      <c r="K17" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
+      <c r="K18" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
+      <c r="K19" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="K20" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="K21" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="K22" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
+      <c r="K23" s="42" t="s">
+        <v>126</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+      <c r="K24" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="L24" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="K25" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="L25" s="24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="K26" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="K27" s="22"/>
+      <c r="L27" s="22"/>
+    </row>
+    <row r="28" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="K28" s="22"/>
+      <c r="L28" s="22"/>
+    </row>
+    <row r="29" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
+      <c r="K29" s="22"/>
+      <c r="L29" s="22"/>
+    </row>
+    <row r="30" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
+      <c r="K30" s="22"/>
+      <c r="L30" s="22"/>
+    </row>
+    <row r="31" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
+      <c r="K31" s="22"/>
+      <c r="L31" s="22"/>
+    </row>
+    <row r="32" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="K32" s="22"/>
+      <c r="L32" s="22"/>
+    </row>
+    <row r="33" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="K33" s="22"/>
+      <c r="L33" s="22"/>
+    </row>
+    <row r="34" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="K34" s="22"/>
+      <c r="L34" s="22"/>
+    </row>
+    <row r="35" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G35" s="22"/>
+      <c r="H35" s="22"/>
+      <c r="K35" s="22"/>
+      <c r="L35" s="22"/>
+    </row>
+    <row r="36" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G36" s="22"/>
+      <c r="H36" s="22"/>
+      <c r="K36" s="22"/>
+      <c r="L36" s="22"/>
+    </row>
+    <row r="37" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G37" s="22"/>
+      <c r="H37" s="22"/>
+      <c r="K37" s="22"/>
+      <c r="L37" s="22"/>
+    </row>
+    <row r="38" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+    </row>
+    <row r="39" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+    </row>
+    <row r="40" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+    </row>
+    <row r="41" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="K41" s="10"/>
+      <c r="L41" s="10"/>
+    </row>
+    <row r="42" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{037F023B-37BE-4680-9FAC-E053276B2DC2}">
+  <dimension ref="G1:L42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="8" width="22.5703125" customWidth="1"/>
+    <col min="11" max="12" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="28" t="s">
+        <v>123</v>
+      </c>
+      <c r="L3" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G4" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G5" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K5" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G6" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K6" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G7" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K7" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G8" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K8" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G9" s="41" t="s">
+        <v>129</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K9" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G10" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K10" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G11" s="20" t="s">
+        <v>101</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K11" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G12" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K12" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G13" s="20" t="s">
+        <v>130</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K13" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G14" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K14" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G15" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K15" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G16" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K16" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G17" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K17" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G18" s="39" t="s">
+        <v>81</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="K18" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G19" s="39" t="s">
+        <v>79</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="K19" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="K20" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G21" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="K21" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K22" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="7:12" ht="131.25" x14ac:dyDescent="0.25">
+      <c r="G23" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="K23" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G24" s="25" t="s">
+        <v>134</v>
+      </c>
+      <c r="H24" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="K24" s="39" t="s">
+        <v>141</v>
+      </c>
+      <c r="L24" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G25" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="H25" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="K25" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="26" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G26" s="27" t="s">
+        <v>137</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K26" s="26" t="s">
+        <v>142</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G27" s="43" t="s">
+        <v>138</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="K27" s="22"/>
+      <c r="L27" s="22"/>
+    </row>
+    <row r="28" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="K28" s="22"/>
+      <c r="L28" s="22"/>
+    </row>
+    <row r="29" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
+      <c r="K29" s="22"/>
+      <c r="L29" s="22"/>
+    </row>
+    <row r="30" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
+      <c r="K30" s="22"/>
+      <c r="L30" s="22"/>
+    </row>
+    <row r="31" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
+      <c r="K31" s="22"/>
+      <c r="L31" s="22"/>
+    </row>
+    <row r="32" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="K32" s="22"/>
+      <c r="L32" s="22"/>
+    </row>
+    <row r="33" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="K33" s="22"/>
+      <c r="L33" s="22"/>
+    </row>
+    <row r="34" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="K34" s="22"/>
+      <c r="L34" s="22"/>
+    </row>
+    <row r="35" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G35" s="22"/>
+      <c r="H35" s="22"/>
+      <c r="K35" s="22"/>
+      <c r="L35" s="22"/>
+    </row>
+    <row r="36" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G36" s="22"/>
+      <c r="H36" s="22"/>
+      <c r="K36" s="22"/>
+      <c r="L36" s="22"/>
+    </row>
+    <row r="37" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G37" s="22"/>
+      <c r="H37" s="22"/>
+      <c r="K37" s="22"/>
+      <c r="L37" s="22"/>
+    </row>
+    <row r="38" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+    </row>
+    <row r="39" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+    </row>
+    <row r="40" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+    </row>
+    <row r="41" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="K41" s="10"/>
+      <c r="L41" s="10"/>
+    </row>
+    <row r="42" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F01B2EE5-E16D-45BB-A8B1-B5ACE9400842}">
+  <dimension ref="G1:L42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="8" width="22.5703125" customWidth="1"/>
+    <col min="11" max="12" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="28" t="s">
+        <v>123</v>
+      </c>
+      <c r="L3" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G4" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G5" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K5" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G6" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K6" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G7" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K7" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G8" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K8" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G9" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K9" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G10" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K10" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G11" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K11" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G12" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K12" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G13" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K13" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G14" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K14" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K15" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K16" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G17" s="26" t="s">
+        <v>76</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K17" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L17" s="24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G18" s="27" t="s">
+        <v>146</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K18" s="11"/>
+      <c r="L18" s="11"/>
+    </row>
+    <row r="19" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G19" s="29" t="s">
+        <v>98</v>
+      </c>
+      <c r="H19" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="K19" s="22"/>
+      <c r="L19" s="22"/>
+    </row>
+    <row r="20" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
+    </row>
+    <row r="21" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="22"/>
+    </row>
+    <row r="22" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="22"/>
+    </row>
+    <row r="23" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="22"/>
+    </row>
+    <row r="24" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+      <c r="K24" s="22"/>
+      <c r="L24" s="22"/>
+    </row>
+    <row r="25" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="K25" s="22"/>
+      <c r="L25" s="22"/>
+    </row>
+    <row r="26" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="K26" s="22"/>
+      <c r="L26" s="22"/>
+    </row>
+    <row r="27" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="K27" s="22"/>
+      <c r="L27" s="22"/>
+    </row>
+    <row r="28" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="K28" s="22"/>
+      <c r="L28" s="22"/>
+    </row>
+    <row r="29" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
+      <c r="K29" s="22"/>
+      <c r="L29" s="22"/>
+    </row>
+    <row r="30" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
+      <c r="K30" s="22"/>
+      <c r="L30" s="22"/>
+    </row>
+    <row r="31" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
+      <c r="K31" s="22"/>
+      <c r="L31" s="22"/>
+    </row>
+    <row r="32" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="K32" s="22"/>
+      <c r="L32" s="22"/>
+    </row>
+    <row r="33" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="K33" s="22"/>
+      <c r="L33" s="22"/>
+    </row>
+    <row r="34" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="K34" s="22"/>
+      <c r="L34" s="22"/>
+    </row>
+    <row r="35" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G35" s="22"/>
+      <c r="H35" s="22"/>
+      <c r="K35" s="22"/>
+      <c r="L35" s="22"/>
+    </row>
+    <row r="36" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G36" s="22"/>
+      <c r="H36" s="22"/>
+      <c r="K36" s="22"/>
+      <c r="L36" s="22"/>
+    </row>
+    <row r="37" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G37" s="22"/>
+      <c r="H37" s="22"/>
+      <c r="K37" s="22"/>
+      <c r="L37" s="22"/>
+    </row>
+    <row r="38" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+    </row>
+    <row r="39" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+    </row>
+    <row r="40" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+    </row>
+    <row r="41" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="K41" s="10"/>
+      <c r="L41" s="10"/>
+    </row>
+    <row r="42" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{400711E2-41E9-4F6A-8D66-AD1A160D8245}">
+  <dimension ref="G1:L42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="8" width="22.5703125" customWidth="1"/>
+    <col min="11" max="12" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="L3" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G4" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K4" s="26" t="s">
+        <v>107</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G5" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K5" s="26" t="s">
+        <v>102</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G6" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K6" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G7" s="26" t="s">
+        <v>145</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K7" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G8" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K8" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G9" s="26" t="s">
+        <v>98</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K9" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G10" s="26" t="s">
+        <v>132</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K10" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G11" s="26" t="s">
+        <v>146</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K11" s="26" t="s">
+        <v>106</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G12" s="26" t="s">
+        <v>95</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K12" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G13" s="44" t="s">
+        <v>147</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K13" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G14" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K14" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G15" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K15" s="26" t="s">
+        <v>97</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G16" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K16" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>148</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G18" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K18" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G19" s="39" t="s">
+        <v>149</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K19" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G20" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K20" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G21" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K21" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="7:12" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="G22" s="39" t="s">
+        <v>150</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K22" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="23" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G23" s="39" t="s">
+        <v>151</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K23" s="46" t="s">
+        <v>153</v>
+      </c>
+      <c r="L23" s="24" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="24" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G24" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="H24" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="K24" s="39" t="s">
+        <v>156</v>
+      </c>
+      <c r="L24" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
+      <c r="K25" s="31"/>
+      <c r="L25" s="31"/>
+    </row>
+    <row r="26" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="K26" s="31"/>
+      <c r="L26" s="31"/>
+    </row>
+    <row r="27" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="K27" s="31"/>
+      <c r="L27" s="31"/>
+    </row>
+    <row r="28" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="K28" s="31"/>
+      <c r="L28" s="31"/>
+    </row>
+    <row r="29" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
+      <c r="K29" s="31"/>
+      <c r="L29" s="31"/>
+    </row>
+    <row r="30" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
+      <c r="K30" s="31"/>
+      <c r="L30" s="31"/>
+    </row>
+    <row r="31" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
+      <c r="K31" s="31"/>
+      <c r="L31" s="31"/>
+    </row>
+    <row r="32" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="K32" s="31"/>
+      <c r="L32" s="31"/>
+    </row>
+    <row r="33" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="K33" s="31"/>
+      <c r="L33" s="31"/>
+    </row>
+    <row r="34" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="K34" s="31"/>
+      <c r="L34" s="31"/>
+    </row>
+    <row r="35" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G35" s="22"/>
+      <c r="H35" s="22"/>
+      <c r="K35" s="31"/>
+      <c r="L35" s="31"/>
+    </row>
+    <row r="36" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G36" s="22"/>
+      <c r="H36" s="22"/>
+      <c r="K36" s="31"/>
+      <c r="L36" s="31"/>
+    </row>
+    <row r="37" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G37" s="22"/>
+      <c r="H37" s="22"/>
+      <c r="K37" s="31"/>
+      <c r="L37" s="31"/>
+    </row>
+    <row r="38" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+    </row>
+    <row r="39" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+    </row>
+    <row r="40" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+    </row>
+    <row r="41" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="K41" s="10"/>
+      <c r="L41" s="10"/>
+    </row>
+    <row r="42" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6152ECF6-CCB6-4201-9459-562479E56238}">
+  <dimension ref="G1:L42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="8" width="22.5703125" customWidth="1"/>
+    <col min="11" max="12" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G3" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="34" t="s">
+        <v>110</v>
+      </c>
+      <c r="L3" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G4" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K4" s="27" t="s">
+        <v>92</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G5" s="38" t="s">
+        <v>157</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K5" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G6" s="38" t="s">
+        <v>158</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K6" s="27" t="s">
+        <v>102</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G7" s="32" t="s">
+        <v>118</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K7" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G8" s="32" t="s">
+        <v>103</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K8" s="27" t="s">
+        <v>91</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G9" s="32" t="s">
+        <v>132</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K9" s="27" t="s">
+        <v>82</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G10" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K10" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G11" s="27" t="s">
+        <v>122</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K11" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G12" s="27" t="s">
+        <v>130</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K12" s="27" t="s">
+        <v>167</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G13" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K13" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G14" s="27" t="s">
+        <v>159</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K14" s="43" t="s">
+        <v>168</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G15" s="43" t="s">
+        <v>160</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K15" s="27" t="s">
+        <v>169</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G16" s="27" t="s">
+        <v>161</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K16" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G17" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G18" s="39" t="s">
+        <v>162</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K18" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G19" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K19" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G20" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K20" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G21" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K21" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G22" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K22" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G23" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K23" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G24" s="26" t="s">
+        <v>139</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K24" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="L24" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G25" s="26" t="s">
+        <v>134</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K25" s="33" t="s">
+        <v>152</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G26" s="26" t="s">
+        <v>164</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K26" s="11"/>
+      <c r="L26" s="11"/>
+    </row>
+    <row r="27" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G27" s="26" t="s">
+        <v>183</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K27" s="22"/>
+      <c r="L27" s="22"/>
+    </row>
+    <row r="28" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G28" s="44" t="s">
+        <v>165</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K28" s="22"/>
+      <c r="L28" s="22"/>
+    </row>
+    <row r="29" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G29" s="45" t="s">
+        <v>166</v>
+      </c>
+      <c r="H29" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="K29" s="22"/>
+      <c r="L29" s="22"/>
+    </row>
+    <row r="30" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G30" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K30" s="22"/>
+      <c r="L30" s="22"/>
+    </row>
+    <row r="31" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K31" s="22"/>
+      <c r="L31" s="22"/>
+    </row>
+    <row r="32" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="K32" s="22"/>
+      <c r="L32" s="22"/>
+    </row>
+    <row r="33" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="K33" s="22"/>
+      <c r="L33" s="22"/>
+    </row>
+    <row r="34" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="K34" s="22"/>
+      <c r="L34" s="22"/>
+    </row>
+    <row r="35" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G35" s="22"/>
+      <c r="H35" s="22"/>
+      <c r="K35" s="22"/>
+      <c r="L35" s="22"/>
+    </row>
+    <row r="36" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G36" s="22"/>
+      <c r="H36" s="22"/>
+      <c r="K36" s="22"/>
+      <c r="L36" s="22"/>
+    </row>
+    <row r="37" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G37" s="22"/>
+      <c r="H37" s="22"/>
+      <c r="K37" s="22"/>
+      <c r="L37" s="22"/>
+    </row>
+    <row r="38" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+    </row>
+    <row r="39" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+    </row>
+    <row r="40" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+    </row>
+    <row r="41" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="K41" s="10"/>
+      <c r="L41" s="10"/>
+    </row>
+    <row r="42" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33AE33F0-FC25-41A5-B62E-B291D044B50E}">
+  <dimension ref="G1:L42"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="8" width="22.5703125" customWidth="1"/>
+    <col min="11" max="12" width="22.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="7:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="7:12" ht="47.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" spans="7:12" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G3" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="K3" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="L3" s="15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G4" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K4" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G5" s="39" t="s">
+        <v>170</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K5" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G6" s="39" t="s">
+        <v>171</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K6" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G7" s="39" t="s">
+        <v>172</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G8" s="35" t="s">
+        <v>89</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K8" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G9" s="40" t="s">
+        <v>173</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K9" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G10" s="35" t="s">
+        <v>122</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K10" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G11" s="35" t="s">
+        <v>85</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K11" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G12" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K12" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G13" s="42" t="s">
+        <v>175</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K13" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G14" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K14" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G15" s="42" t="s">
+        <v>177</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K15" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G16" s="42" t="s">
+        <v>178</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K16" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G17" s="44" t="s">
+        <v>180</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K17" s="14" t="s">
+        <v>100</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G18" s="44" t="s">
+        <v>181</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K18" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G19" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K19" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G20" s="20" t="s">
+        <v>159</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K20" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G21" s="20" t="s">
+        <v>183</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K21" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G22" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K22" s="36" t="s">
+        <v>140</v>
+      </c>
+      <c r="L22" s="24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="7:12" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="G23" s="41" t="s">
+        <v>182</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K23" s="11"/>
+      <c r="L23" s="11"/>
+    </row>
+    <row r="24" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G24" s="20" t="s">
+        <v>139</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K24" s="22"/>
+      <c r="L24" s="22"/>
+    </row>
+    <row r="25" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G25" s="32" t="s">
+        <v>145</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K25" s="22"/>
+      <c r="L25" s="22"/>
+    </row>
+    <row r="26" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G26" s="32" t="s">
+        <v>148</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="K26" s="22"/>
+      <c r="L26" s="22"/>
+    </row>
+    <row r="27" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G27" s="36" t="s">
+        <v>134</v>
+      </c>
+      <c r="H27" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="K27" s="22"/>
+      <c r="L27" s="22"/>
+    </row>
+    <row r="28" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="K28" s="22"/>
+      <c r="L28" s="22"/>
+    </row>
+    <row r="29" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
+      <c r="K29" s="22"/>
+      <c r="L29" s="22"/>
+    </row>
+    <row r="30" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
+      <c r="K30" s="22"/>
+      <c r="L30" s="22"/>
+    </row>
+    <row r="31" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
+      <c r="K31" s="22"/>
+      <c r="L31" s="22"/>
+    </row>
+    <row r="32" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="K32" s="22"/>
+      <c r="L32" s="22"/>
+    </row>
+    <row r="33" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="K33" s="22"/>
+      <c r="L33" s="22"/>
+    </row>
+    <row r="34" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="K34" s="22"/>
+      <c r="L34" s="22"/>
+    </row>
+    <row r="35" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G35" s="22"/>
+      <c r="H35" s="22"/>
+      <c r="K35" s="22"/>
+      <c r="L35" s="22"/>
+    </row>
+    <row r="36" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G36" s="22"/>
+      <c r="H36" s="22"/>
+      <c r="K36" s="22"/>
+      <c r="L36" s="22"/>
+    </row>
+    <row r="37" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G37" s="22"/>
+      <c r="H37" s="22"/>
+      <c r="K37" s="22"/>
+      <c r="L37" s="22"/>
+    </row>
+    <row r="38" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K38" s="10"/>
+      <c r="L38" s="10"/>
+    </row>
+    <row r="39" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="K39" s="10"/>
+      <c r="L39" s="10"/>
+    </row>
+    <row r="40" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+    </row>
+    <row r="41" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="K41" s="10"/>
+      <c r="L41" s="10"/>
+    </row>
+    <row r="42" spans="7:12" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>